<commit_message>
feat: implement admin availability management, time range slots, and admin logout functionality
</commit_message>
<xml_diff>
--- a/bookings_export.xlsx
+++ b/bookings_export.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:N4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -436,6 +436,12 @@
       <c r="L1" t="str">
         <v>Created At</v>
       </c>
+      <c r="M1" t="str">
+        <v>Updated At</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Cancellation Reason</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -504,15 +510,65 @@
         <v>1</v>
       </c>
       <c r="J3" t="str">
-        <v>cancelled</v>
+        <v>completed</v>
+      </c>
+      <c r="K3" t="str">
+        <v xml:space="preserve"> [Reactivated on 3/16/2026]</v>
       </c>
       <c r="L3" t="str">
         <v>2026-03-14T17:06:13.243Z</v>
+      </c>
+      <c r="M3" t="str">
+        <v>2026-03-16T08:03:08.117Z</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>pt-0003</v>
+      </c>
+      <c r="B4" t="str">
+        <v>2026-03-18</v>
+      </c>
+      <c r="C4" t="str">
+        <v>3:00 PM</v>
+      </c>
+      <c r="D4" t="str">
+        <v>abu</v>
+      </c>
+      <c r="E4" t="str">
+        <v>0771123456</v>
+      </c>
+      <c r="F4" t="str">
+        <v>toyota sbvu (2000)</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Engine Tune-Up</v>
+      </c>
+      <c r="H4">
+        <v>15000</v>
+      </c>
+      <c r="I4">
+        <v>3</v>
+      </c>
+      <c r="J4" t="str">
+        <v>completed</v>
+      </c>
+      <c r="K4" t="str">
+        <v>tuneup [Reactivated on 3/16/2026]</v>
+      </c>
+      <c r="L4" t="str">
+        <v>2026-03-16T07:38:20.061Z</v>
+      </c>
+      <c r="M4" t="str">
+        <v>2026-03-16T08:03:07.519Z</v>
+      </c>
+      <c r="N4" t="str">
+        <v>cancel due to customer bc</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>